<commit_message>
Add tariff verification of proposed code 4412999090
The customer proposed reclassifying to 4412999090. Verified it against
the goods using the CCT/VPV KN method from the reference deck.

Conclusion: the code does not match the invoice description. Heading
4412 splits first on whether the panel consists solely of sheets of
wood each not exceeding 6 mm. All documents describe plywood, and item
3 is a 4 mm panel, which cannot contain a ply over 6 mm, so the 4412 9x
branch is excluded. The manufacturer also declares 441233 himself.

Correct code depends on the species of both outer plies; if both are
coniferous it is 4412 39 00 at 7% with no anti-dumping, which is
cheaper than the 10% the customer offered to pay.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVghCknMruivM8JHkAAeLW
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
+++ b/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
@@ -10,6 +10,7 @@
     <sheet name="HS Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Položky faktury (rozpad)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Dokumenty a poznámky" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ověření HS 4412999090" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +38,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +68,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -151,6 +161,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1560,4 +1579,568 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A85"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="145" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>OVĚŘENÍ NAVRŽENÉHO KÓDU 4412 99 90 90 — postup dle CCT/VPV KN tariff rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Podnět: zákazník (Area Four Industries) dne 22.9.2026 sdělil, že kód 4412331082 je omyl a žádá proclení pod 4412999090</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>s odůvodněním, že „pod tímto číslem bylo vždycky cleno v minulosti“ a s odkazem na interní e-mail MW ze 17.12.2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Metodika: reference/Common_Customs_Tariff_EU_CZ.pptx, slide 18–19 (tři zbožíznalecké otázky + VPV KN 1–6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>POZN.: Nejde o odvození chybějícího kódu — kód byl dodán. Jde o ověření, zda navržený kód odpovídá zboží.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>KROK 1 — TŘI ZBOŽÍZNALECKÉ OTÁZKY</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>CO TO JE? — Překližkové desky (plywood), formátované, povrchově upravené hnědým fenolickým filmem Dynea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pět rozměrů, celková tloušťka desky 4 / 12 / 15 / 18 mm. Jedna strana hladký film, druhá protiskluzový rastr</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   („honeycomb wire mesh“ = vzor filmu, NIKOLI voštinové jádro). U pol. 4 je jedna strana bez filmu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Z ČEHO TO JE? — Dřevěné dýhové listy spojené lepidlem Dynea (fenolická pryskyřice). Lícová dýha borovice</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   („PINE FACED“ = jehličnatá dřevina). Dřevina rubové dýhy a jádra není v dokladech uvedena — JEDINÝ CHYBĚJÍCÍ ÚDAJ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>K ČEMU SLOUŽÍ? — Konstrukční deska; u Area Four (pódiové a trusové systémy) typicky pódiové a bednicí desky.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>KROK 2 — TŘÍDA, KAPITOLA, POZNÁMKY</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Třída IX — Dřevo a dřevěné výrobky. Kapitola 44 — Dřevo a dřevěné výrobky; dřevěné uhlí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Úvodní poznámky ke kap. 44 zboží nevylučují. Podle VPV 1 → číslo 4412 „Překližky, dýhované desky a podobné vrstvené dřevo“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Číslo 4412 je pro obě porovnávané varianty společné — spor se rozhoduje až na úrovni položek (VPV 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>KROK 3 — ROZHODUJÍCÍ DĚLENÍ UVNITŘ ČÍSLA 4412 (VPV 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Číslo 4412 se dělí nejprve takto:</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 10          — z bambusu</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ► „Ostatní překližky, sestávající pouze z dřevěných listů (jiných než bambusových),</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      o tloušťce každé vrstvy NEPŘESAHUJÍCÍ 6 mm:“  → 4412 31 / 4412 33 / 4412 34 / 4412 39</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ► „Ostatní:“ → vrstvené dřevo, které do předchozí skupiny NEPATŘÍ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      4412 41/42/49 — vrstvené dýhové dřevo (LVL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      4412 51/52/59 — laťovky, spárovky (blockboard, laminboard, battenboard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      4412 91/92/99 — ostatní   →   4412 99 = „Ostatní, s oběma vnějšími vrstvami z jehličnatého dřeva“</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                     →   4412 99 90 90 = „Ostatní“ (navržený kód)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>JEDINÉ KRITÉRIUM, které tyto dvě větve odděluje, zní: sestává deska POUZE z dřevěných listů,</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>z nichž ŽÁDNÝ nepřesahuje 6 mm? ANO → 4412 3x. NE → 4412 4x/5x/9x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Kritérium se NEtýká celkové tloušťky desky, nýbrž tloušťky JEDNOTLIVÉ VRSTVY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>KROK 4 — APLIKACE KRITÉRIA NA NAŠE ZBOŽÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>a) Všechny doklady (faktura RH-26-048S, packing list, shipment advice, COO, B/L) popisují zboží shodně</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   jako „PLYWOOD“ — tedy překližku z dýhových listů, nikoli laťovku, LVL ani desku s dřevotřískovým jádrem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>b) DŮKAZ, KTERÝ NELZE VYVRÁTIT: položka 3 je deska 4 × 993 × 1993 mm. Celková tloušťka desky jsou 4 mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   V desce silné 4 mm nemůže být vrstva přesahující 6 mm. U této položky je 4412 99 vyloučené absolutně.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>c) Filmový povrch na zařazení nic nemění — povrchová úprava je v textu podpoložek výslovně připuštěna</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   („whether or not coated or surface-covered“) a neruší podmínku „sestávající pouze z dřevěných listů“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>d) Sám výrobce uvádí na faktuře, B/L i certifikátu původu HS 441233 — tedy kód ze skupiny do 6 mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Je to prohlášení výrobce o vlastním výrobku a svědčí proti zařazení do 4412 9x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="inlineStr">
+        <is>
+          <t>ZÁVĚR: KÓD 4412 99 90 90 NEODPOVÍDÁ POPISU ZBOŽÍ NA FAKTUŘE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="25" t="inlineStr">
+        <is>
+          <t>Popis zboží navržený kód nepodporuje — naopak ho aktivně vylučuje. Podle VPV 1 a VPV 6 patří zboží</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>do skupiny „pouze z dřevěných listů do 6 mm“, tedy do 4412 31 / 33 / 34 / 39.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>Kód 4412 99 90 90 by byl správný POUZE tehdy, pokud by deska obsahovala vrstvu silnější než 6 mm nebo</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>nedřevěnou/nedýhovou vrstvu, a zároveň nešlo o LVL ani laťovku. Nic takového z dokladů neplyne</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>a u 4 mm desky je to fyzicky nemožné. Pokud takovou skladbu výrobce doloží, zařazení se přehodnotí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="23" t="inlineStr">
+        <is>
+          <t>KROK 5 — SPRÁVNÝ KÓD ZÁVISÍ NA DŘEVINĚ VNĚJŠÍCH DÝH</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>Uvnitř skupiny do 6 mm rozhoduje dřevina vnějších vrstev:</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 31        — alespoň jedna vnější vrstva z tropického dřeva ......................... nepřichází v úvahu</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 33 10     — alespoň jedna vnější vrstva BŘÍZA ......... clo 7 % + ANTIDUMPING 86,8 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 33 20     — alespoň jedna vnější vrstva TOPOL/OSIKA ... clo 7 % + ANTIDUMPING 86,8 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 33 30     — alespoň jedna vnější vrstva EUKALYPTUS .... clo 7 % + ANTIDUMPING 86,8 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 33 90     — jiná dřevina ze seznamu 4412 33 ........... clo 7 % + ANTIDUMPING 86,8 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 34        — jiné listnaté dřevo ....................... clo 7 % + ANTIDUMPING 86,8 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 39 00     — OBĚ vnější vrstvy JEHLIČNATÉ ............. clo 7 %, BEZ ANTIDUMPINGU</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>Doklady uvádějí „PINE FACED“, tedy borovicovou LÍCOVOU dýhu. Chybí údaj o RUBOVÉ dýze.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>Jsou-li obě vnější dýhy jehličnaté → 4412 39 00 (TARIC 4412390020), clo 7 %, antidumping se neuplatní.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>Pozor: nařízení (EU) 2025/2333 dává TARIC 4412390020 výslovně pod monitoring Komise jako možný obcházecí</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>scénář, takže toto zařazení musí být doloženo technickým listem výrobce, ne pouze tvrzením.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="23" t="inlineStr">
+        <is>
+          <t>SROVNÁNÍ VARIANT (základ US $33 839,84 + dopravné do hranice EU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 39 00 00   clo 7 %,  bez AD ....................... cca US $2 369    ← pokud jsou obě dýhy borovicové</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 99 90 90   clo 10 %, bez AD ...................... cca US $3 384    ← navrhuje zákazník, popisu neodpovídá</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   4412 33 10 82   clo 7 % + AD 86,8 % ................... cca US $31 742   ← původně zadaný kód</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>POZNÁMKA: zákazník si říká o variantu, která je i v případě její správnosti DRAŽŠÍ než legitimní 4412 39 00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="23" t="inlineStr">
+        <is>
+          <t>K ARGUMENTU „VŽDYCKY SE TAK CLILO“</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>Podle slide 19 referenčního decku a ustálené judikatury SDEU jsou rozhodujícím kritériem pro sazební zařazení</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>OBJEKTIVNÍ CHARAKTERISTIKY ZBOŽÍ — složení a zamýšlené použití — jak je vymezuje znění podpoložek KN</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>a poznámky ke třídě/kapitole. Dosavadní praxe ani dřívější celní prohlášení zařazení nezakládají.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>Minulé zásilky mohly mít jinou skladbu desky, a pak byl kód správný. Pokud šlo o totéž zboží, jsou dotčené také —</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>doměření podle čl. 103 UCC běží tři roky zpětně.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="22" t="inlineStr">
+        <is>
+          <t>CO JE TŘEBA DOLOŽIT PŘED PODÁNÍM JSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>Technický list výrobce (Xuzhou Lara) s údaji: dřevina lícové dýhy, dřevina rubové dýhy, dřevina jádra,</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="inlineStr">
+        <is>
+          <t>počet vrstev a tloušťka jednotlivých vrstev. Tento jediný dokument rozhodne mezi všemi třemi variantami výše.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>Při přetrvávající pochybnosti eskalovat na tarifní tým: customs.tariff@mauriceward.com (slide 23).</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="inlineStr">
+        <is>
+          <t>Do budoucna doporučuji zákazníkovi požádat o ZIS (závaznou informaci o sazebním zařazení) — vyřízení cca 120 dní.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Split Area Four CZ26011062 into final HS codes per customer instruction
Per Lukas Jirkovsky's instruction of 9 Oct 2026 (clear according to the
customer's item split, confirmed by Marcela Kirilova):

- 4412 33 10 82: GM5-Deska 4 x 993 x 1993 mm, 518 sheets, NW 2,620 kg,
  GW 2,680 kg, USD 189.00; definitive AD duty 86.8%.
- 4412 39 00 30: the other four items, 1,968 sheets, NW 35,300 kg,
  GW 36,050 kg, USD 33,650.84; 7%, no definitive AD, imports registered
  under Reg. 2026/1840.

Totals still reconcile to the invoice and B/L. Flags that the customer's
table lists only 18 sheets of the 4 mm board while the documents show
518 (500 free of charge), and that the FOC sheets need a customs value.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVghCknMruivM8JHkAAeLW
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
+++ b/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,10 +37,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="7">
@@ -62,12 +58,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -102,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -119,10 +115,22 @@
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -139,39 +147,31 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -537,22 +537,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="78" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -568,7 +569,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Popis dle dokladů (EN)</t>
+          <t>Položky dle zákazníka (Reg. č. – Název 3)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -593,7 +594,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Objem (m³)</t>
+          <t>Objem (m³) – MJ MTQ</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -613,16 +614,21 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Clo / opatření</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Příznak</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Poznámka / TARIC / CBAM / Antidumping</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="150" customHeight="1">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>4412 33 10 82</t>
@@ -635,13 +641,14 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>PINE FACED PLYWOOD – one side honeycomb wire mesh smooth Dynea brown film / one side smooth Dynea brown film, other side no film / both side smooth Dynea brown film; Dynea glue. 5 rozměrů, 27 beden.</t>
+          <t>39201508 – GM5-Deska 993x1993x4 Hexa-VOP
+(faktura: 4 × 993 × 1993 mm – 18 ks à $10,50 + 500 ks FREE OF CHARGE)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>RILICO GLOBAL HOLDINGS PTE LTD, 111 Somerset Road #15-18, Singapore 238164
-(výrobce dle COO: XUZHOU LARA IMPORT &amp; EXPORT CO., LTD, Pizhou City, Jiangsu, ČLR)</t>
+(výrobce dle COO: XUZHOU LARA IMPORT &amp; EXPORT CO., LTD, Pizhou, Jiangsu, ČLR)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -655,129 +662,199 @@
         </is>
       </c>
       <c r="G2" s="3" t="n">
+        <v>518</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>4.101</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>2620</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>2680</v>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>189</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>7 % + konečné AD clo 86,8 % (nař. (EU) 2025/2333), doplňkový kód 8999</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>ANTIDUMPING / FOC 500 ks</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Kód dle pokynu zákazníka (9.10.2026): „V minulosti clili pod AD, prosím toto zopakovat.“
+⚠ Zákazník v tabulce uvádí jen 18 ks – faktura i packing list mají 518 ks (500 ks zdarma). Bezúplatné listy patří do JSD s celní hodnotou a podléhají také AD clu – viz list „Dokumenty a poznámky“, bod 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="135" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>4412 39 00 30</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Popis zboží v češtině zákazník nedodal – uvedeny jeho názvy položek (viz vedlejší sloupec).</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>30207943 – Plywood birch/pine 1994x994x12 hexa 220 (S10-Deska)
+39200442 – SM-STAIR-Woodplate 910x225x15
+21200058 – Poplar plywood 18x1220x2440mm (both sides Dynea film)
+39201550 – Plywood birch/pine 1993x993x15 hexa 220 with hole</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>RILICO GLOBAL HOLDINGS PTE LTD, 111 Somerset Road #15-18, Singapore 238164
+(výrobce dle COO: XUZHOU LARA IMPORT &amp; EXPORT CO., LTD, Pizhou, Jiangsu, ČLR)</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>CN (Čína)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>FOB Qingdao (Qingdao Port, Čína)</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>1968</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>54.026</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>35300</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>36050</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>33650.84</v>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>7 %, BEZ konečného AD cla; registrace dovozu dle nař. (EU) 2026/1840 (od 25.7.2026) + statistické sledování dle 2026/822</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>AD REGISTRACE</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Zařazení potvrdila tarifní specialistka V. Šimůnková (30.9.2026): překližka pouze z dýh ≤ 6 mm, obě vnější dýhy borovice &lt; 2,5 mm, jádro bříza + topol → 4412390030. Skladbu písemně potvrdil M. Jiskra (A4I, 30.9.2026).
+⚠ Registrace dovozu: potvrdí-li šetření obcházení AD opatření, lze AD clo uplatnit ZPĚTNĚ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>CELKEM</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr"/>
+      <c r="C4" s="10" t="inlineStr"/>
+      <c r="D4" s="10" t="inlineStr"/>
+      <c r="E4" s="10" t="inlineStr"/>
+      <c r="F4" s="10" t="inlineStr"/>
+      <c r="G4" s="11" t="n">
         <v>2486</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H4" s="12" t="n">
         <v>58.127</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="I4" s="11" t="n">
         <v>37920</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="J4" s="11" t="n">
         <v>38730</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K4" s="13" t="n">
         <v>33839.84</v>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>ANTIDUMPING / OVĚŘIT KLASIFIKACI</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>⚠ ANTIDUMPING: TARIC 4412331082 je ve věcném rozsahu prov. nařízení Komise (EU) 2025/2333 (tvrdá překližka z ČLR, platnost 21.11.2025–20.11.2030) – konečné AD clo 86,8 % (43,2 % pro jednoho spolupracujícího vývozce). Xuzhou Lara není známa jako vývozce s individuální sazbou → hrozí 86,8 %.
-⚠ KLASIFIKACE: doklady uvádějí PINE FACED (jehličnatá dýha), e-mail/klient uvádí 4412331082 = alespoň jedna vnější dýha BŘÍZA. Nutno ověřit dřevinu obou vnějších dýh (viz list „Dokumenty a poznámky“).
-CBAM: NEAPLIKUJE SE – kap. 44 není zboží dle přílohy I nařízení o CBAM.
-EUDR: 4412 je v příloze I nař. (EU) 2023/1115, ale použitelnost od 30.12.2026 → pro toto celní řízení (9–10/2026) se DDS/Y-kód nevyžaduje.
-Clo (CCT): 7 % erga omnes – ověřit v TARIC k datu propuštění.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>CELKEM</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="7" t="n">
-        <v>2486</v>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>58.127</v>
-      </c>
-      <c r="I3" s="7" t="n">
-        <v>37920</v>
-      </c>
-      <c r="J3" s="7" t="n">
-        <v>38730</v>
-      </c>
-      <c r="K3" s="9" t="n">
-        <v>33839.84</v>
-      </c>
-      <c r="L3" s="6" t="inlineStr"/>
-      <c r="M3" s="6" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="L4" s="10" t="inlineStr"/>
+      <c r="M4" s="10" t="inlineStr"/>
+      <c r="N4" s="10" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Legenda:</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>🔴 ČERVENÁ</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Antidumpingové clo a/nebo nevyjasněná sazební klasifikace – nutno vyřešit PŘED podáním JSD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Množství</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>2 486 listů celkem (vč. 500 listů FREE OF CHARGE) / 58,127 m³ / 27 beden / 1×20'GP + 1×40'HQ.</t>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Konečné antidumpingové clo – uvést v JSD.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>🟡 ORANŽOVÁ</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Bez konečného AD cla, ale dovoz je registrován (nař. 2026/1840) – riziko zpětného AD cla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Zdroj kódů</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Pokyn L. Jirkovského 9.10.2026 16:20: „prosím tedy o vyclení dle instrukcí zákazníka“ (tabulka zákazníka z 8.10.2026); M. Kirilova 9.10.2026: „máme vyclít tak, jak je níže od nich psáno, je to jejich volba“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Cena</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Použita částka u položky „TOTAL“ na faktuře RH-26-048S: US $33 839,84 (bez přičítání hodnoty FOC listů).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Částky ze sloupce TOTAL AMOUNT faktury RH-26-048S po položkách; součet = TOTAL US $33 839,84.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Hmotnosti</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Dle Packing/Weight List – NW 37 920 kg, GW 38 730 kg; ověřeno součtem po bednách i dle B/L.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>Popis CZ</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Převzat klientský český popis „březová překližka“ z pokynu (e-mail OR/AREA FOUR/KLI20260701011/CZ26011062) – viz výhrada na listu poznámek.</t>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Packing/Weight List po bednách, sečteno po HS kódech; součty sedí na NW 37 920 kg / GW 38 730 kg i B/L.</t>
         </is>
       </c>
     </row>
@@ -792,18 +869,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -814,224 +893,286 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Popis / rozměr</t>
+          <t>Popis dle faktury / rozměr</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Reg. č. zákazníka</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>HS kód (TARIC)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Listů</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Objem (m³)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Beden</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>NW (kg)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>GW (kg)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Jedn. cena USD/list</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Celkem USD</t>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Celkem USD (TOTAL AMOUNT)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="n">
+      <c r="A2" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>Pine faced plywood, one side honeycomb wire mesh smooth Dynea brown film, Dynea glue – 15 × 993 × 1993 mm</t>
         </is>
       </c>
-      <c r="C2" s="13" t="n">
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>39201550</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>4412 39 00 30</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="n">
         <v>496</v>
       </c>
-      <c r="D2" s="14" t="n">
+      <c r="F2" s="18" t="n">
         <v>14.724</v>
       </c>
-      <c r="E2" s="12" t="n">
+      <c r="G2" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="F2" s="13" t="n">
+      <c r="H2" s="17" t="n">
         <v>9430</v>
       </c>
-      <c r="G2" s="13" t="n">
+      <c r="I2" s="17" t="n">
         <v>9640</v>
       </c>
-      <c r="H2" s="15" t="n">
+      <c r="J2" s="19" t="n">
         <v>20.79</v>
       </c>
-      <c r="I2" s="15" t="n">
+      <c r="K2" s="19" t="n">
         <v>10311.84</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n">
+      <c r="A3" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>Pine faced plywood, one side honeycomb wire mesh smooth Dynea brown film, Dynea glue – 12 × 994 × 1994 mm</t>
         </is>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>30207943</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>4412 39 00 30</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="n">
         <v>494</v>
       </c>
-      <c r="D3" s="14" t="n">
+      <c r="F3" s="18" t="n">
         <v>11.75</v>
       </c>
-      <c r="E3" s="12" t="n">
+      <c r="G3" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="H3" s="17" t="n">
         <v>7880</v>
       </c>
-      <c r="G3" s="13" t="n">
+      <c r="I3" s="17" t="n">
         <v>8090</v>
       </c>
-      <c r="H3" s="15" t="n">
+      <c r="J3" s="19" t="n">
         <v>17.95</v>
       </c>
-      <c r="I3" s="15" t="n">
+      <c r="K3" s="19" t="n">
         <v>8867.299999999999</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Pine faced plywood, one side honeycomb wire mesh smooth Dynea brown film, Dynea glue – 4 × 993 × 1993 mm (18 ks à $10,50 + 500 ks FREE OF CHARGE)</t>
         </is>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>39201508</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>4412 33 10 82</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>518</v>
       </c>
-      <c r="D4" s="14" t="n">
+      <c r="F4" s="4" t="n">
         <v>4.101</v>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="G4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="13" t="n">
+      <c r="H4" s="3" t="n">
         <v>2620</v>
       </c>
-      <c r="G4" s="13" t="n">
+      <c r="I4" s="3" t="n">
         <v>2680</v>
       </c>
-      <c r="H4" s="15" t="n">
+      <c r="J4" s="5" t="n">
         <v>10.5</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="K4" s="5" t="n">
         <v>189</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Pine faced plywood, one side smooth Dynea brown film, other side no film, Dynea glue – 15 × 225 × 910 mm</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>39200442</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>4412 39 00 30</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="n">
         <v>492</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="F5" s="18" t="n">
         <v>1.511</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="G5" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="H5" s="17" t="n">
         <v>970</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="I5" s="17" t="n">
         <v>1000</v>
       </c>
-      <c r="H5" s="15" t="n">
+      <c r="J5" s="19" t="n">
         <v>2.2</v>
       </c>
-      <c r="I5" s="15" t="n">
+      <c r="K5" s="19" t="n">
         <v>1082.4</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Pine faced plywood, both side smooth Dynea brown film, Dynea glue – 18 × 1220 × 2440 mm</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>21200058</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>4412 39 00 30</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="n">
         <v>486</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="F6" s="18" t="n">
         <v>26.041</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="G6" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="H6" s="17" t="n">
         <v>17020</v>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="I6" s="17" t="n">
         <v>17320</v>
       </c>
-      <c r="H6" s="15" t="n">
+      <c r="J6" s="19" t="n">
         <v>27.55</v>
       </c>
-      <c r="I6" s="15" t="n">
+      <c r="K6" s="19" t="n">
         <v>13389.3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr"/>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr"/>
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>CELKEM (TOTAL dle faktury)</t>
         </is>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="20" t="inlineStr"/>
+      <c r="D7" s="20" t="inlineStr"/>
+      <c r="E7" s="21" t="n">
         <v>2486</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="F7" s="22" t="n">
         <v>58.127</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="G7" s="21" t="n">
         <v>27</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="H7" s="21" t="n">
         <v>37920</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="I7" s="21" t="n">
         <v>38730</v>
       </c>
-      <c r="H7" s="20" t="inlineStr"/>
-      <c r="I7" s="20" t="n">
+      <c r="J7" s="23" t="inlineStr"/>
+      <c r="K7" s="23" t="n">
         <v>33839.84</v>
       </c>
     </row>
@@ -1046,533 +1187,395 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A80"/>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="140" customWidth="1" min="1" max="1"/>
+    <col width="145" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21">
+      <c r="A1" s="24">
         <f>== ZÁSILKA ===</f>
         <v/>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Klient / příjemce (CZ): AREA FOUR INDUSTRIES ČESKO s.r.o., Spindlerova třída 286, CZ 413 01 Roudnice nad Labem | DIČ/EORI CZ25003330</t>
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Příjemce: AREA FOUR INDUSTRIES ČESKO s.r.o., Spindlerova třída 286, CZ 413 01 Roudnice nad Labem | EORI CZ25003330</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Odesílatel / vývozce: RILICO GLOBAL HOLDINGS PTE LTD, Singapur | Výrobce (dle COO): XUZHOU LARA IMPORT &amp; EXPORT CO., LTD, Pizhou City, Jiangsu, ČLR</t>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Odesílatel: RILICO GLOBAL HOLDINGS PTE LTD, Singapur | Výrobce (dle COO): XUZHOU LARA IMPORT &amp; EXPORT CO., LTD, Pizhou, Jiangsu, ČLR</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Faktura: RH-26-048S z 31.7.2026 | Objednávky: P-021225-TC &amp; P-010226-TC | Ref. MW: CZ26011062 / KLI20260701011</t>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Faktura RH-26-048S z 31.7.2026 | Objednávky P-021225-TC &amp; P-010226-TC | Ref. MW CZ26011062 / KLI20260701011</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>B/L: F202616848 (Global Transportation Agency Ltd.), shipped on board 28.7.2026, vystaveno Shantou | Loď: MV MAASTRICHT MAERSK / 630W</t>
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>B/L F202616848 (kopie) | MV MAERSK MAASTRICHT / 630W | Qingdao → Bremerhaven → Mělník | FOB Qingdao Port | freight collect</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Trasa: FOB Qingdao Port (ČLR) → Bremerhaven → Mělník (ČR), freight collect, platba T/T | ATA Bremerhaven 8.9.2026</t>
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Kontejnery: MRKU8681136 / CN7598690 – 10 beden | MRSU2171077 / CN6068214 – 17 beden | celkem 27 beden, 2 486 listů, 58,127 m³</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Kontejnery: MRKU8681136 / seal CN7598690 – 10 beden / 12 130 kg / 17,925 m³ ; MRSU2171077 / seal CN6068214 – 17 beden / 26 600 kg / 40,202 m³</t>
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Režim: volný oběh (40), bez AZS – potvrdil L. Jirkovský 23.9.2026. JSD přes Mělník, MRN pošle P. Vojtěchová.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Celkem: 27 beden, 2 486 listů, 58,127 m³, NW 37 920 kg, GW 38 730 kg, hodnota US $33 839,84</t>
-        </is>
-      </c>
+      <c r="A8" s="15" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr"/>
+      <c r="A9" s="25">
+        <f>== FINÁLNÍ ZAŘAZENÍ – dle pokynu zákazníka (L. Jirkovský, 9.10.2026 16:20) ===</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="22">
-        <f>== ⚠ 1. ANTIDUMPINGOVÉ CLO – KRITICKÉ ===</f>
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Zákazník (tabulka z 8.10.2026) rozdělil položky takto, M. Kirilova (9.10.2026) potvrdila: „je to jejich volba, celní úřad bude spokojen“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   39201508  GM5-Deska 993x1993x4 Hexa-VOP ............................ 4412 33 10 82   (zákazník: „V minulosti clili pod AD, prosím toto zopakovat“)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   30207943  Plywood birch/pine 1994x994x12 hexa 220 (S10-Deska) ........ 4412 39 00 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   39200442  SM-STAIR-Woodplate 910x225x15 ............................. 4412 39 00 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   21200058  Poplar plywood 18x1220x2440mm (both sides Dynea film) ...... 4412 39 00 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   39201550  Plywood birch/pine 1993x993x15 hexa 220 with hole .......... 4412 39 00 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Podklad pro 4412390030: V. Šimůnková 30.9.2026 – překližka pouze z dýh ≤ 6 mm, obě vnější dýhy borovice (Pinus) &lt; 2,5 mm,</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   jádro bříza + topol. Skladbu potvrdil písemně M. Jiskra (A4I) 30.9.2026 9:22 a 9:47. Žádná dřevotříska, vrstvy cca do 5 mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Kódy 4412999090 a původní celoplošný 4412331082 jsou tímto nahrazeny (historie viz list „Ověření HS 4412999090“).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="26">
+        <f>== ⚠ 1. ANTIDUMPING – 4412 33 10 82 (GM5-Deska 4 mm) ===</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Prov. nařízení Komise (EU) 2025/2333 z 19.11.2025 uložilo KONEČNÉ antidumpingové clo na tvrdou překližku (hardwood plywood) původem z ČLR,</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>platné od 21.11.2025 do 20.11.2030. Sazba: 86,8 % pro všechny vývozce, 43,2 % pro jednoho spolupracujícího vývozce.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Věcný rozsah zahrnuje mj. TARIC 4412331082 – tedy přesně kód uvedený v pokynu klienta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>Výrobce Xuzhou Lara Import &amp; Export Co., Ltd sídlí v Pizhou (Jiangsu) – hlavní oblast, na kterou opatření cílí; firma není známa jako vývozce s individuální sazbou.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>→ Při klasifikaci do 4412331082 činí AD clo cca US $29 372 (86,8 % z 33 839,84) NAD RÁMEC běžného cla. Nutno klienta upozornit PŘED propuštěním.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>→ Ověřit v TARIC doplňkový kód TARIC pro výrobce a případné osvobození; doložit fakturu výrobce a prohlášení dle čl. o individuální sazbě.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="22">
-        <f>== ⚠ 2. ROZPOR V SAZEBNÍM ZAŘAZENÍ – NUTNO VYJASNIT ===</f>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Konečné AD clo 86,8 % dle nař. (EU) 2025/2333 (21.11.2025–20.11.2030), doplňkový kód 8999 (všechny ostatní společnosti) + clo 7 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Z fakturované částky US $189,00 → AD cca US $164,05 + clo cca US $13,23 (bez dopravného a bez hodnoty FOC listů – viz bod 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="26">
+        <f>== ⚠ 2. 500 LISTŮ „FREE OF CHARGE“ – CHYBÍ V TABULCE ZÁKAZNÍKA ===</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>Všechny doklady (faktura, packing list, COO, B/L, shipment advice) popisují zboží jako „PINE FACED PLYWOOD“ – tj. borovicová (JEHLIČNATÁ) vnější dýha.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Pokyn klienta v e-mailu však uvádí kód 4412331082 s popisem „březová překližka“ (BŘÍZA = listnatá dřevina).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Doklady odesílatele uvádějí pouze šestimístné „HS CODE: 441233“, což samo o sobě podpoložku 4412 33 10 (bříza) nepotvrzuje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Rozhodující je dřevina OBOU vnějších dýh:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   a) alespoň jedna vnější dýha bříza → 4412 33 10 (TARIC 4412331082) → AD clo 86,8 % (viz bod 1);</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   b) alespoň jedna vnější dýha jiná listnatá dřevina ze seznamu 4412 33 (topol, osika…) → 4412 33 90 10 → rovněž v rozsahu AD opatření;</t>
-        </is>
-      </c>
-    </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   c) OBĚ vnější dýhy jehličnaté (borovice) s listnatým jádrem → 4412 39 00, TARIC 4412390020 – MIMO AD clo, ale nařízení 2025/2333 tento kód</t>
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Tabulka zákazníka uvádí u 39201508 jen 18 ks. Faktura, packing list i COO ale mají u rozměru 4 × 993 × 1993 mm 518 listů</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      výslovně podrobuje MONITORINGU Komise právě jako možný obcházecí („modified product“) scénář; clo 7 %.</t>
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (18 ks à $10,50 = $189,00 + 500 ks FREE OF CHARGE), 2 bedny, 4,101 m³, NW 2 620 kg, GW 2 680 kg.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>→ Vyžádat od klienta/výrobce specifikaci skladby desky (dřevina lícové i rubové dýhy a jádra), ideálně technický list nebo prohlášení výrobce.</t>
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>V souhrnu je proto 518 listů – jinak by nesouhlasil celkový počet 2 486 listů ani hmotnosti s B/L.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>→ Vzhledem k rozdílu 7 % vs. 86,8 % doporučuji před podáním JSD konzultovat sazební oddělení: customs.tariff@mauriceward.com.</t>
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Bezúplatné zboží musí být v JSD s celní hodnotou (nelze nulovou). Při ceně $10,50/list jde o cca US $5 250,</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>→ Bez vyjasnění nelze kód odpovědně potvrdit; popis „PINE FACED“ u kódu pro břízu je typický rizikový profil pro celní kontrolu.</t>
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   z čehož AD 86,8 % ≈ US $4 557 + clo 7 % ≈ US $368. → Potvrdit se zákazníkem hodnotu FOC listů PŘED podáním JSD.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr"/>
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Pozn.: Dle pravidla „Total“ je ve sloupci ceny uvedena jen fakturovaná částka $189,00 – hodnota FOC listů v ní NENÍ.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="23">
-        <f>== 3. ODPOVĚĎ NA DOTAZ: „Je k HS kódu vyžadován Y-code?“ ===</f>
+      <c r="A31" s="15" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="27">
+        <f>== ⚠ 3. 4412 39 00 30 – REGISTRACE DOVOZU (bez konečného AD cla) ===</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>a) CBAM Y-kódy (Y128 / Y238 / Y137): NE. CBAM se vztahuje pouze na zboží přílohy I nařízení (EU) 2023/956 – cement, elektřina, hnojiva,</t>
-        </is>
-      </c>
-    </row>
     <row r="33">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   železo a ocel, hliník, vodík (kap. 25, 27, 28, 31, 72, 73, 76). Překližka kap. 44 mezi ně nepatří → žádný CBAM Y-kód se neuvádí.</t>
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>Clo 7 %. Konečné AD clo zatím není, ale dovoz podléhá registraci dle nař. (EU) 2026/1840 (od 25.7.2026) a statistickému</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   (Pro pořádek: příjemce Area Four Industries Česko s.r.o. JE v naší evidenci CBAM – viz bod 4 – ale pro tuto zásilku je to bezpředmětné.)</t>
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   sledování dle nař. (EU) 2026/822. Potvrdí-li šetření obcházení AD opatření, může být AD clo na registrované dovozy uplatněno ZPĚTNĚ.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>b) EUDR (nařízení (EU) 2023/1115, odlesňování): kód 4412 JE v příloze I nařízení. Použitelnost však byla nařízením (EU) 2025/2650</t>
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (zdroj: V. Šimůnková, 30.9.2026) → doporučeno upozornit zákazníka, že riziko není uzavřené.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   odložena na 30.12.2026 pro velké a střední subjekty (30.6.2027 pro mikro a malé). Toto celní řízení proběhne v 9–10/2026,</t>
-        </is>
-      </c>
+      <c r="A36" s="15" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   tedy PŘED tímto datem → DDS (kód dokladu C716) ani Y-kód EUDR se zatím nevyžaduje.</t>
-        </is>
+      <c r="A37" s="27">
+        <f>== ⚠ 4. NÁZVY POLOŽEK ZÁKAZNÍKA vs. ZAŘAZENÍ ===</f>
+        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   → Upozornit klienta, že od 30.12.2026 bude pro každou další dodávku překližky nutné prohlášení o náležité péči (DDS) s geolokací.</t>
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>Položka 21200058 se v systému zákazníka jmenuje „Poplar plywood …“ a položky 30207943 / 39201550 „Plywood birch/pine …“,</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>c) Sankce vůči Rusku (nař. 833/2014, příloha XXI zahrnuje kap. 44): původ je ČLR, doložen COO. Ověřit v TARIC k datu propuštění, zda je</t>
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   faktura u všech uvádí „PINE FACED PLYWOOD“. Pro 4412 39 rozhodují jen VNĚJŠÍ dýhy; zákazník písemně potvrdil, že obě vnější</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   u konkrétního kódu vyžadován prohlašovací Y-kód o neruském původu; pokud ano, doložit důkaz o původu.</t>
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   jsou borovice a bříza/topol jsou v jádru. Názvy tomu nemusí odporovat, ale u kontroly mohou vzbudit otázky →</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>→ SHRNUTÍ pro klienta: CBAM Y-kód se NEVYŽADUJE; EUDR zatím také ne (až od 30.12.2026). Skutečným problémem není Y-kód, ale ANTIDUMPING (bod 1).</t>
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   doporučeno popis v JSD formulovat podle skladby (vnější dýhy borovice, jádro bříza/topol), ne podle názvu „Poplar plywood“.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="inlineStr"/>
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Zároveň: 4mm GM5-Deska má na faktuře rovněž „PINE FACED“, zákazník ji ale sám deklaruje jako březovou (4412331082) – jeho volba,</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="21">
-        <f>== 4. CBAM – LOOKUP PŘÍJEMCE (reference/CBAM_receivers_CZ.xlsx, list List1) ===</f>
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   z hlediska cla jde o přísnější (dražší) variantu, riziko doměření nevzniká.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="24">
+        <f>== 5. CBAM / EUDR / OCEL ===</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>Příjemce NALEZEN v registru:</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Firma: Area Four Industries Česko s.r.o.</t>
-        </is>
-      </c>
-    </row>
     <row r="46">
-      <c r="A46" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   EORI: CZ25003330</t>
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>CBAM: neaplikuje se (kap. 44 není zboží přílohy I). Příjemce je v registru: Area Four Industries Česko s.r.o., EORI CZ25003330,</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Y KÓD: Y238 (podaná žádost, dosud neschválený deklarant)</t>
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Y238, žádost APPL-CZ-2026-WTI716839226323 – pro tuto zásilku bez významu. Sdílený účet CBAM-CZ-2025-QGM67089385721: netýká se.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Podaná žádost: APPL-CZ-2026-WTI716839226323 (prověřeno k 8.7. – Marcela_kontejner CAIU4695926)</t>
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>EUDR: 4412 je v příloze I nař. (EU) 2023/1115, použitelnost od 30.12.2026 → u tohoto proclení DDS nevyžadováno.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Povolení (Y128): – (žádné)   |   Y137 (do 50 t ročně): –   |   Datum vydání: neuvedeno</t>
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Melt and pour: neaplikuje se – zásilka neobsahuje železo ani ocel.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="inlineStr">
-        <is>
-          <t>POZNÁMKA: Tato zásilka NEOBSAHUJE CBAM zboží (překližka kap. 44), takže se Y238 v tomto JSD neuplatní.</t>
-        </is>
-      </c>
+      <c r="A50" s="15" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="11" t="inlineStr">
-        <is>
-          <t>Údaj uvádím pouze pro úplnost – status příjemce je v pořádku a připraven pro budoucí zásilky CBAM zboží.</t>
-        </is>
+      <c r="A51" s="24">
+        <f>== 6. PREFERENČNÍ PŮVOD A REX ===</f>
+        <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="11" t="inlineStr">
-        <is>
-          <t>Zásilka se NETÝKÁ sdíleného účtu CBAM-CZ-2025-QGM67089385721 (Area Four není mezi firmami mimo EU, které jej využívají).</t>
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>PREFERENČNÍ VĚTA: NENALEZENA v žádném dokladu. ČLR nemá s EU preferenční dohodu → kód preference 100, plné třetizemní clo.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="11" t="inlineStr"/>
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>REX ČÍSLO: NA FAKTUŘE NENÍ. Ani číslo celního povolení vývozce v dokladech není.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="23">
-        <f>== 5. PREFERENČNÍ PŮVOD (preferenční věta) A REX ===</f>
+      <c r="A54" s="15" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="24">
+        <f>== 7. DOKLADY ===</f>
         <v/>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>PREFERENČNÍ VĚTA: NENALEZENA v žádném z dokladů (faktura RH-26-048S, packing list, shipment advice, COO, B/L).</t>
-        </is>
-      </c>
-    </row>
     <row r="56">
-      <c r="A56" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ČLR nemá s EU preferenční dohodu, takže preferenční zacházení stejně nepřichází v úvahu – uplatní se plné třetizemní clo (CCT 7 %).</t>
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>✓ Faktura RH-26-048S, ✓ Packing/Weight List, ✓ Shipment Advice – vše 31.7.2026, vzájemně souhlasí.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Faktura naopak obsahuje pouze prohlášení, že zboží je „wholly of Chinese origin“ a „not of Israeli origin“ – to NENÍ preferenční věta.</t>
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>⚠ B/L F202616848 jen kopie „NOT NEGOTIABLE“ – pro výdej originál nebo D/O.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="inlineStr">
-        <is>
-          <t>REX ČÍSLO: NA FAKTUŘE NENÍ UVEDENO. Výslovně konstatuji jeho nepřítomnost.</t>
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>⚠ COO (Singapur) jen DRAFT bez čísla, podpisu a razítka; příjemce chybně „AREA FOUR INDUSTRIES ESKO S.R.O.“.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Žádné číslo REX ani číslo celního povolení vývozce se v dokladech nevyskytuje. Vzhledem k původu ČLR to nemá dopad na clo,</t>
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>⚠ FOB Qingdao → do celní hodnoty připočíst dopravu a pojištění do místa vstupu do EU (vyžádat přepravní fakturu).</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   protože nárok na preferenci by stejně nevznikl. Pro zařazení do spisu je však absence zaznamenána.</t>
+      <c r="A60" s="15" t="inlineStr">
+        <is>
+          <t>Sleva: na faktuře žádná – proporcionální rozpad slevy se neuplatní.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="21">
-        <f>== 6. DOKLADY – STAV A ZÁVADY ===</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="11" t="inlineStr">
-        <is>
-          <t>✓ Commercial Invoice RH-26-048S (31.7.2026) – obsahuje položku „TOTAL“ US $33 839,84, použita jako celní hodnota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="11" t="inlineStr">
-        <is>
-          <t>✓ Packing / Weight List (31.7.2026) – hmotnosti po bednách, souhlasí s fakturou i B/L.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="11" t="inlineStr">
-        <is>
-          <t>✓ Shipment Advice (31.7.2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="11" t="inlineStr">
-        <is>
-          <t>✓ Bill of Lading F202616848 – kopie „NOT NEGOTIABLE – COPY“. Pro propuštění bude třeba originál B/L nebo Delivery Order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="11" t="inlineStr">
-        <is>
-          <t>⚠ Certificate of Origin (Singapore) – pouze ve stavu „DRAFT“, BEZ čísla, BEZ podpisu a BEZ razítka příslušného orgánu (pole 12 nevyplněno).</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   → Vyžádat vystavený a ověřený originál COO. Při AD opatření je doklad o původu zásadní.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>⚠ V COO je příjemce uveden chybně jako „AREA FOUR INDUSTRIES ESKO S.R.O.“ (chybí Č v „ČESKO“) → nechat opravit při vystavení originálu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="11" t="inlineStr">
-        <is>
-          <t>⚠ 500 listů je na faktuře uvedeno jako „FREE OF CHARGE“ (rozměr 4 × 993 × 1993 mm). Dle pokynu je do souhrnu převzata částka „TOTAL“,</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   tedy bez dopočtu hodnoty FOC listů. Pro celní hodnotu je však nutné cenu bezúplatně dodaného zboží doložit/dopočítat –</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   při jednotkové ceně $10,50/list by šlo o cca US $5 250. → Vyjasnit s klientem, zda má být tato částka do celní hodnoty zahrnuta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="11" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="21">
-        <f>== 7. DALŠÍ ===</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="11" t="inlineStr">
-        <is>
-          <t>Incoterm: FOB Qingdao Port, Čína (uveden shodně na faktuře, shipment advice i COO). Do celní hodnoty je proto nutné připočíst</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   náklady na dopravu a pojištění do místa vstupu do EU (freight collect – vyžádat přepravní fakturu).</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="11" t="inlineStr">
-        <is>
-          <t>Obchodní sleva: na faktuře NENÍ uvedena žádná sleva (žádný subtotal/discount/before-after discount) → proporcionální rozpad slevy se neuplatní.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="11" t="inlineStr">
-        <is>
-          <t>Sazební zařazení nebylo odvozováno postupem „CCT/VPV KN tariff rule“ – HS kód byl v podkladech dodán (441233 / 4412331082);</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   předmětem je jeho OVĚŘENÍ, nikoli odvození. Viz bod 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="11" t="inlineStr">
-        <is>
-          <t>JSD: přes Mělník (Maersk), vyclení do volného oběhu.</t>
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>Zařazení nebylo odvozováno postupem „CCT/VPV KN tariff rule“ – kódy dodal zákazník a potvrdila tarifní specialistka MW.</t>
         </is>
       </c>
     </row>
@@ -1587,554 +1590,561 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A85"/>
+  <dimension ref="A1:A86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="145" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>HISTORIE (22.–25.9.2026): ověření návrhu 4412999090 – zamítnuto. Konečné zařazení viz list „HS Summary“.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>OVĚŘENÍ NAVRŽENÉHO KÓDU 4412 99 90 90 — postup dle CCT/VPV KN tariff rule</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Podnět: zákazník (Area Four Industries) dne 22.9.2026 sdělil, že kód 4412331082 je omyl a žádá proclení pod 4412999090</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>s odůvodněním, že „pod tímto číslem bylo vždycky cleno v minulosti“ a s odkazem na interní e-mail MW ze 17.12.2025.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Metodika: reference/Common_Customs_Tariff_EU_CZ.pptx, slide 18–19 (tři zbožíznalecké otázky + VPV KN 1–6).</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>POZN.: Nejde o odvození chybějícího kódu — kód byl dodán. Jde o ověření, zda navržený kód odpovídá zboží.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr"/>
-    </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="15" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>KROK 1 — TŘI ZBOŽÍZNALECKÉ OTÁZKY</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>CO TO JE? — Překližkové desky (plywood), formátované, povrchově upravené hnědým fenolickým filmem Dynea.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Pět rozměrů, celková tloušťka desky 4 / 12 / 15 / 18 mm. Jedna strana hladký film, druhá protiskluzový rastr</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   („honeycomb wire mesh“ = vzor filmu, NIKOLI voštinové jádro). U pol. 4 je jedna strana bez filmu.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Z ČEHO TO JE? — Dřevěné dýhové listy spojené lepidlem Dynea (fenolická pryskyřice). Lícová dýha borovice</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   („PINE FACED“ = jehličnatá dřevina). Dřevina rubové dýhy a jádra není v dokladech uvedena — JEDINÝ CHYBĚJÍCÍ ÚDAJ.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>K ČEMU SLOUŽÍ? — Konstrukční deska; u Area Four (pódiové a trusové systémy) typicky pódiové a bednicí desky.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="15" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>KROK 2 — TŘÍDA, KAPITOLA, POZNÁMKY</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Třída IX — Dřevo a dřevěné výrobky. Kapitola 44 — Dřevo a dřevěné výrobky; dřevěné uhlí.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Úvodní poznámky ke kap. 44 zboží nevylučují. Podle VPV 1 → číslo 4412 „Překližky, dýhované desky a podobné vrstvené dřevo“.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Číslo 4412 je pro obě porovnávané varianty společné — spor se rozhoduje až na úrovni položek (VPV 6).</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr"/>
-    </row>
     <row r="20">
-      <c r="A20" s="23" t="inlineStr">
+      <c r="A20" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>KROK 3 — ROZHODUJÍCÍ DĚLENÍ UVNITŘ ČÍSLA 4412 (VPV 6)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Číslo 4412 se dělí nejprve takto:</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 10          — z bambusu</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   ► „Ostatní překližky, sestávající pouze z dřevěných listů (jiných než bambusových),</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">      o tloušťce každé vrstvy NEPŘESAHUJÍCÍ 6 mm:“  → 4412 31 / 4412 33 / 4412 34 / 4412 39</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   ► „Ostatní:“ → vrstvené dřevo, které do předchozí skupiny NEPATŘÍ:</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">      4412 41/42/49 — vrstvené dýhové dřevo (LVL)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">      4412 51/52/59 — laťovky, spárovky (blockboard, laminboard, battenboard)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">      4412 91/92/99 — ostatní   →   4412 99 = „Ostatní, s oběma vnějšími vrstvami z jehličnatého dřeva“</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">                                     →   4412 99 90 90 = „Ostatní“ (navržený kód)</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="15" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>JEDINÉ KRITÉRIUM, které tyto dvě větve odděluje, zní: sestává deska POUZE z dřevěných listů,</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>z nichž ŽÁDNÝ nepřesahuje 6 mm? ANO → 4412 3x. NE → 4412 4x/5x/9x.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>Kritérium se NEtýká celkové tloušťky desky, nýbrž tloušťky JEDNOTLIVÉ VRSTVY.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="11" t="inlineStr"/>
-    </row>
     <row r="35">
-      <c r="A35" s="23" t="inlineStr">
+      <c r="A35" s="15" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>KROK 4 — APLIKACE KRITÉRIA NA NAŠE ZBOŽÍ</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>a) Všechny doklady (faktura RH-26-048S, packing list, shipment advice, COO, B/L) popisují zboží shodně</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   jako „PLYWOOD“ — tedy překližku z dýhových listů, nikoli laťovku, LVL ani desku s dřevotřískovým jádrem.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>b) DŮKAZ, KTERÝ NELZE VYVRÁTIT: položka 3 je deska 4 × 993 × 1993 mm. Celková tloušťka desky jsou 4 mm.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   V desce silné 4 mm nemůže být vrstva přesahující 6 mm. U této položky je 4412 99 vyloučené absolutně.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>c) Filmový povrch na zařazení nic nemění — povrchová úprava je v textu podpoložek výslovně připuštěna</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   („whether or not coated or surface-covered“) a neruší podmínku „sestávající pouze z dřevěných listů“.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>d) Sám výrobce uvádí na faktuře, B/L i certifikátu původu HS 441233 — tedy kód ze skupiny do 6 mm.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="11" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Je to prohlášení výrobce o vlastním výrobku a svědčí proti zařazení do 4412 9x.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="11" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="A45" s="22" t="inlineStr">
+      <c r="A45" s="15" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>ZÁVĚR: KÓD 4412 99 90 90 NEODPOVÍDÁ POPISU ZBOŽÍ NA FAKTUŘE.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="25" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>Popis zboží navržený kód nepodporuje — naopak ho aktivně vylučuje. Podle VPV 1 a VPV 6 patří zboží</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="25" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>do skupiny „pouze z dřevěných listů do 6 mm“, tedy do 4412 31 / 33 / 34 / 39.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="11" t="inlineStr"/>
-    </row>
     <row r="49">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="A49" s="15" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>Kód 4412 99 90 90 by byl správný POUZE tehdy, pokud by deska obsahovala vrstvu silnější než 6 mm nebo</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="11" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr">
         <is>
           <t>nedřevěnou/nedýhovou vrstvu, a zároveň nešlo o LVL ani laťovku. Nic takového z dokladů neplyne</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>a u 4 mm desky je to fyzicky nemožné. Pokud takovou skladbu výrobce doloží, zařazení se přehodnotí.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="11" t="inlineStr"/>
-    </row>
     <row r="53">
-      <c r="A53" s="23" t="inlineStr">
+      <c r="A53" s="15" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>KROK 5 — SPRÁVNÝ KÓD ZÁVISÍ NA DŘEVINĚ VNĚJŠÍCH DÝH</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="11" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="15" t="inlineStr">
         <is>
           <t>Uvnitř skupiny do 6 mm rozhoduje dřevina vnějších vrstev:</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 31        — alespoň jedna vnější vrstva z tropického dřeva ......................... nepřichází v úvahu</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="11" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 33 10     — alespoň jedna vnější vrstva BŘÍZA ......... clo 7 % + ANTIDUMPING 86,8 %</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 33 20     — alespoň jedna vnější vrstva TOPOL/OSIKA ... clo 7 % + ANTIDUMPING 86,8 %</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 33 30     — alespoň jedna vnější vrstva EUKALYPTUS .... clo 7 % + ANTIDUMPING 86,8 %</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 33 90     — jiná dřevina ze seznamu 4412 33 ........... clo 7 % + ANTIDUMPING 86,8 %</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 34        — jiné listnaté dřevo ....................... clo 7 % + ANTIDUMPING 86,8 %</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="26" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 39 00     — OBĚ vnější vrstvy JEHLIČNATÉ ............. clo 7 %, BEZ ANTIDUMPINGU</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="11" t="inlineStr"/>
-    </row>
     <row r="63">
-      <c r="A63" s="11" t="inlineStr">
+      <c r="A63" s="15" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>Doklady uvádějí „PINE FACED“, tedy borovicovou LÍCOVOU dýhu. Chybí údaj o RUBOVÉ dýze.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="11" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="15" t="inlineStr">
         <is>
           <t>Jsou-li obě vnější dýhy jehličnaté → 4412 39 00 (TARIC 4412390020), clo 7 %, antidumping se neuplatní.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="11" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="15" t="inlineStr">
         <is>
           <t>Pozor: nařízení (EU) 2025/2333 dává TARIC 4412390020 výslovně pod monitoring Komise jako možný obcházecí</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="11" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
         <is>
           <t>scénář, takže toto zařazení musí být doloženo technickým listem výrobce, ne pouze tvrzením.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="11" t="inlineStr"/>
-    </row>
     <row r="68">
-      <c r="A68" s="23" t="inlineStr">
+      <c r="A68" s="15" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
         <is>
           <t>SROVNÁNÍ VARIANT (základ US $33 839,84 + dopravné do hranice EU)</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 39 00 00   clo 7 %,  bez AD ....................... cca US $2 369    ← pokud jsou obě dýhy borovicové</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="11" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 99 90 90   clo 10 %, bez AD ...................... cca US $3 384    ← navrhuje zákazník, popisu neodpovídá</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="11" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   4412 33 10 82   clo 7 % + AD 86,8 % ................... cca US $31 742   ← původně zadaný kód</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="11" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
         <is>
           <t>POZNÁMKA: zákazník si říká o variantu, která je i v případě její správnosti DRAŽŠÍ než legitimní 4412 39 00.</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="11" t="inlineStr"/>
-    </row>
     <row r="74">
-      <c r="A74" s="23" t="inlineStr">
+      <c r="A74" s="15" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="15" t="inlineStr">
         <is>
           <t>K ARGUMENTU „VŽDYCKY SE TAK CLILO“</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="11" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="15" t="inlineStr">
         <is>
           <t>Podle slide 19 referenčního decku a ustálené judikatury SDEU jsou rozhodujícím kritériem pro sazební zařazení</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="11" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="15" t="inlineStr">
         <is>
           <t>OBJEKTIVNÍ CHARAKTERISTIKY ZBOŽÍ — složení a zamýšlené použití — jak je vymezuje znění podpoložek KN</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="11" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="15" t="inlineStr">
         <is>
           <t>a poznámky ke třídě/kapitole. Dosavadní praxe ani dřívější celní prohlášení zařazení nezakládají.</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="11" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="15" t="inlineStr">
         <is>
           <t>Minulé zásilky mohly mít jinou skladbu desky, a pak byl kód správný. Pokud šlo o totéž zboží, jsou dotčené také —</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="11" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="15" t="inlineStr">
         <is>
           <t>doměření podle čl. 103 UCC běží tři roky zpětně.</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="11" t="inlineStr"/>
-    </row>
     <row r="81">
-      <c r="A81" s="22" t="inlineStr">
+      <c r="A81" s="15" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="15" t="inlineStr">
         <is>
           <t>CO JE TŘEBA DOLOŽIT PŘED PODÁNÍM JSD</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="11" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="15" t="inlineStr">
         <is>
           <t>Technický list výrobce (Xuzhou Lara) s údaji: dřevina lícové dýhy, dřevina rubové dýhy, dřevina jádra,</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="11" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="15" t="inlineStr">
         <is>
           <t>počet vrstev a tloušťka jednotlivých vrstev. Tento jediný dokument rozhodne mezi všemi třemi variantami výše.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="11" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="15" t="inlineStr">
         <is>
           <t>Při přetrvávající pochybnosti eskalovat na tarifní tým: customs.tariff@mauriceward.com (slide 23).</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="11" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="15" t="inlineStr">
         <is>
           <t>Do budoucna doporučuji zákazníkovi požádat o ZIS (závaznou informaci o sazebním zařazení) — vyřízení cca 120 dní.</t>
         </is>

</xml_diff>

<commit_message>
Add split into two customs declarations for CZ26011062
JSD 1 carries everything invoiced (4412 39 00 30 plus the 18 paid 4 mm
sheets under 4412 33 10 82, together USD 33,839.84). JSD 2 carries the
500 free-of-charge 4 mm sheets under 4412 33 10 82 at an assumed
USD 10.50 per sheet, pending the customer's confirmation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVghCknMruivM8JHkAAeLW
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
+++ b/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="HS Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Položky faktury (rozpad)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Dokumenty a poznámky" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Ověření HS 4412999090" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Rozdělení na 2 JSD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Položky faktury (rozpad)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dokumenty a poznámky" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Ověření HS 4412999090" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -98,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -172,6 +173,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -869,6 +876,398 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>JSD</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Pol.</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>HS kód (TARIC)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Položka zákazníka</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Listů</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Objem m³ (MTQ)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Beden</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>NW (kg)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>GW (kg)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Hodnota USD</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Základ CZK (orient.)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>A00 clo 7 % (CZK)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>A30 AD 86,8 % (CZK)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Celkem clo + AD (CZK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>JSD 1 – fakturované zboží</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>4412 39 00 30</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>30207943, 39200442, 21200058, 39201550</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="n">
+        <v>1968</v>
+      </c>
+      <c r="F2" s="18" t="n">
+        <v>54.026</v>
+      </c>
+      <c r="G2" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="H2" s="19" t="n">
+        <v>35300</v>
+      </c>
+      <c r="I2" s="19" t="n">
+        <v>36050</v>
+      </c>
+      <c r="J2" s="19" t="n">
+        <v>33650.84</v>
+      </c>
+      <c r="K2" s="17" t="n">
+        <v>719131</v>
+      </c>
+      <c r="L2" s="17" t="n">
+        <v>50339</v>
+      </c>
+      <c r="M2" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="17" t="n">
+        <v>50339</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>JSD 1 – fakturované zboží</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>4412 33 10 82</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>39201508 GM5-Deska 4 mm – 18 placených listů</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>(v 2 bednách s FOC)</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>91.04000000000001</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>93.13</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>189</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>4039</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>283</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>3506</v>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>3789</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>JSD 1 CELKEM</t>
+        </is>
+      </c>
+      <c r="B4" s="20" t="inlineStr"/>
+      <c r="C4" s="20" t="inlineStr"/>
+      <c r="D4" s="20" t="inlineStr"/>
+      <c r="E4" s="21" t="n">
+        <v>1986</v>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>54.169</v>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="H4" s="23" t="n">
+        <v>35391.04</v>
+      </c>
+      <c r="I4" s="23" t="n">
+        <v>36143.13</v>
+      </c>
+      <c r="J4" s="23" t="n">
+        <v>33839.84</v>
+      </c>
+      <c r="K4" s="21" t="n">
+        <v>723170</v>
+      </c>
+      <c r="L4" s="21" t="n">
+        <v>50622</v>
+      </c>
+      <c r="M4" s="21" t="n">
+        <v>3506</v>
+      </c>
+      <c r="N4" s="21" t="n">
+        <v>54128</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>JSD 2 – FREE OF CHARGE</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>4412 33 10 82</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>39201508 GM5-Deska 4 mm – 500 listů zdarma</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>3.958</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>2528.96</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>2586.87</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>5250</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>112194</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>7854</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>97385</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>105238</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>CELKEM ZÁSILKA</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr"/>
+      <c r="C6" s="20" t="inlineStr"/>
+      <c r="D6" s="20" t="inlineStr"/>
+      <c r="E6" s="21" t="n">
+        <v>2486</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>58.127</v>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>27</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>37920</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>38730</v>
+      </c>
+      <c r="J6" s="23" t="inlineStr">
+        <is>
+          <t>33 839,84 + FOC 5 250,00</t>
+        </is>
+      </c>
+      <c r="K6" s="21" t="n">
+        <v>835364</v>
+      </c>
+      <c r="L6" s="21" t="n">
+        <v>58476</v>
+      </c>
+      <c r="M6" s="21" t="n">
+        <v>100891</v>
+      </c>
+      <c r="N6" s="21" t="n">
+        <v>159366</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Poznámky:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>• Rozdělení: JSD 1 = vše fakturované (transakční hodnota, součet = TOTAL faktury US $33 839,84); JSD 2 = 500 listů FREE OF CHARGE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>• Hodnota FOC: 500 × $10,50 (cena stejné desky z faktury) = $5 250 – NUTNO POTVRDIT se zákazníkem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>• CZK přepočteny stejným poměrem jako výpočet K. Lukianové u 18 listů ($189,00 → 4 039 CZK, tj. 21,37037 CZK/USD) – orientační.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>• FOB Qingdao: do základu je ještě třeba připočíst dopravu a pojištění do místa vstupu do EU – částky výše je NEOBSAHUJÍ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>• Hmotnosti 4mm desky: packing list neuvádí rozdělení 18/500 (2 bedny po 259 listech), NW/GW rozpočteny poměrem počtu listů.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>• Beden: 18 placených listů je fyzicky ve stejných 2 bednách jako FOC listy – bedny vykázány jen jednou (JSD 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>• AD clo uvádět zvlášť jako A30 (86,8 %), A00 je jen clo 7 %. DPH (B00) není zahrnuta.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1181,7 +1580,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1584,7 +1983,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add gross/net weight split per transit MRN for CZ26011062
Allocates each declaration item's weights to the two transit MRNs
(20' MRKU8681136: 12,130 kg GW; 40' MRSU2171077: 26,600 kg GW), using
the crate-to-container allocation derived from weights and volumes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVghCknMruivM8JHkAAeLW
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
+++ b/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -173,12 +173,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -547,20 +545,20 @@
   <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" style="30" min="1" max="1"/>
+    <col width="24" customWidth="1" style="30" min="2" max="2"/>
+    <col width="44" customWidth="1" style="30" min="3" max="3"/>
+    <col width="34" customWidth="1" style="30" min="4" max="4"/>
+    <col width="11" customWidth="1" style="30" min="5" max="5"/>
+    <col width="22" customWidth="1" style="30" min="6" max="6"/>
+    <col width="12" customWidth="1" style="30" min="7" max="7"/>
+    <col width="12" customWidth="1" style="30" min="8" max="8"/>
+    <col width="12" customWidth="1" style="30" min="9" max="9"/>
+    <col width="12" customWidth="1" style="30" min="10" max="10"/>
+    <col width="15" customWidth="1" style="30" min="11" max="11"/>
+    <col width="34" customWidth="1" style="30" min="12" max="12"/>
+    <col width="18" customWidth="1" style="30" min="13" max="13"/>
+    <col width="60" customWidth="1" style="30" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -635,7 +633,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="120" customHeight="1">
+    <row r="2" ht="120" customHeight="1" s="30">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>4412 33 10 82</t>
@@ -700,7 +698,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="135" customHeight="1">
+    <row r="3" ht="135" customHeight="1" s="30">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>4412 39 00 30</t>
@@ -798,7 +796,7 @@
       <c r="N4" s="10" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Legenda:</t>
         </is>
@@ -806,7 +804,7 @@
       <c r="B6" s="15" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>🔴 ČERVENÁ</t>
         </is>
@@ -818,7 +816,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>🟡 ORANŽOVÁ</t>
         </is>
@@ -830,7 +828,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Zdroj kódů</t>
         </is>
@@ -842,7 +840,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Cena</t>
         </is>
@@ -854,7 +852,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Hmotnosti</t>
         </is>
@@ -876,23 +874,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" style="30" min="1" max="1"/>
+    <col width="5" customWidth="1" style="30" min="2" max="2"/>
+    <col width="14" customWidth="1" style="30" min="3" max="3"/>
+    <col width="34" customWidth="1" style="30" min="4" max="4"/>
+    <col width="8" customWidth="1" style="30" min="5" max="5"/>
+    <col width="10" customWidth="1" style="30" min="6" max="6"/>
+    <col width="10" customWidth="1" style="30" min="7" max="7"/>
+    <col width="11" customWidth="1" style="30" min="8" max="8"/>
+    <col width="11" customWidth="1" style="30" min="9" max="9"/>
+    <col width="13" customWidth="1" style="30" min="10" max="10"/>
+    <col width="13" customWidth="1" style="30" min="11" max="11"/>
+    <col width="12" customWidth="1" style="30" min="12" max="12"/>
+    <col width="13" customWidth="1" style="30" min="13" max="13"/>
+    <col width="14" customWidth="1" style="30" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1209,51 +1207,261 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>• Rozdělení: JSD 1 = vše fakturované (transakční hodnota, součet = TOTAL faktury US $33 839,84); JSD 2 = 500 listů FREE OF CHARGE.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>• Hodnota FOC: 500 × $10,50 (cena stejné desky z faktury) = $5 250 – NUTNO POTVRDIT se zákazníkem.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>• CZK přepočteny stejným poměrem jako výpočet K. Lukianové u 18 listů ($189,00 → 4 039 CZK, tj. 21,37037 CZK/USD) – orientační.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>• FOB Qingdao: do základu je ještě třeba připočíst dopravu a pojištění do místa vstupu do EU – částky výše je NEOBSAHUJÍ.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>• Hmotnosti 4mm desky: packing list neuvádí rozdělení 18/500 (2 bedny po 259 listech), NW/GW rozpočteny poměrem počtu listů.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>• Beden: 18 placených listů je fyzicky ve stejných 2 bednách jako FOC listy – bedny vykázány jen jednou (JSD 2).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>• AD clo uvádět zvlášť jako A30 (86,8 %), A00 je jen clo 7 %. DPH (B00) není zahrnuta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>ROZPAD HMOTNOSTÍ PODLE MRN / KONTEJNERŮ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>JSD / položka</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr"/>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>HS kód</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr"/>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>GW – MRN …23252J5 (20' MRKU8681136)</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>NW – MRN …23252J5</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>GW – MRN …23258J0 (40' MRSU2171077)</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>NW – MRN …23258J0</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>GW celkem</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="inlineStr">
+        <is>
+          <t>NW celkem</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>JSD 1 / pol. 1</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr"/>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>4412 39 00 30</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr"/>
+      <c r="E19" s="32" t="n">
+        <v>12130</v>
+      </c>
+      <c r="F19" s="32" t="n">
+        <v>11830</v>
+      </c>
+      <c r="G19" s="32" t="n">
+        <v>23920</v>
+      </c>
+      <c r="H19" s="32" t="n">
+        <v>23470</v>
+      </c>
+      <c r="I19" s="32" t="n">
+        <v>36050</v>
+      </c>
+      <c r="J19" s="32" t="n">
+        <v>35300</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>JSD 1 / pol. 2 (18 ks)</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="inlineStr"/>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>4412 33 10 82</t>
+        </is>
+      </c>
+      <c r="D20" s="31" t="inlineStr"/>
+      <c r="E20" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="32" t="n">
+        <v>93.13</v>
+      </c>
+      <c r="H20" s="32" t="n">
+        <v>91.04000000000001</v>
+      </c>
+      <c r="I20" s="32" t="n">
+        <v>93.13</v>
+      </c>
+      <c r="J20" s="32" t="n">
+        <v>91.04000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>JSD 1 CELKEM</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="10" t="inlineStr"/>
+      <c r="E21" s="13" t="n">
+        <v>12130</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>11830</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>24013.13</v>
+      </c>
+      <c r="H21" s="13" t="n">
+        <v>23561.04</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>36143.13</v>
+      </c>
+      <c r="J21" s="13" t="n">
+        <v>35391.04</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>JSD 2 / pol. 1 (500 ks FOC)</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="inlineStr"/>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>4412 33 10 82</t>
+        </is>
+      </c>
+      <c r="D22" s="31" t="inlineStr"/>
+      <c r="E22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="32" t="n">
+        <v>2586.87</v>
+      </c>
+      <c r="H22" s="32" t="n">
+        <v>2528.96</v>
+      </c>
+      <c r="I22" s="32" t="n">
+        <v>2586.87</v>
+      </c>
+      <c r="J22" s="32" t="n">
+        <v>2528.96</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>MRN CELKEM</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr"/>
+      <c r="C23" s="10" t="inlineStr"/>
+      <c r="D23" s="10" t="inlineStr"/>
+      <c r="E23" s="13" t="n">
+        <v>12130</v>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>11830</v>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>26600</v>
+      </c>
+      <c r="H23" s="13" t="n">
+        <v>26090</v>
+      </c>
+      <c r="I23" s="13" t="n">
+        <v>38730</v>
+      </c>
+      <c r="J23" s="13" t="n">
+        <v>37920</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Přiřazení beden ke kontejnerům je odvozeno z hmotností a objemů (doklady ho neuvádějí): 20' = 3 bedny 15×993×1993 + 7 beden 12×994×1994; 40' = zbytek vč. obou beden 4 mm.</t>
         </is>
       </c>
     </row>
@@ -1271,17 +1479,17 @@
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" style="30" min="1" max="1"/>
+    <col width="58" customWidth="1" style="30" min="2" max="2"/>
+    <col width="13" customWidth="1" style="30" min="3" max="3"/>
+    <col width="15" customWidth="1" style="30" min="4" max="4"/>
+    <col width="8" customWidth="1" style="30" min="5" max="5"/>
+    <col width="10" customWidth="1" style="30" min="6" max="6"/>
+    <col width="7" customWidth="1" style="30" min="7" max="7"/>
+    <col width="9" customWidth="1" style="30" min="8" max="8"/>
+    <col width="9" customWidth="1" style="30" min="9" max="9"/>
+    <col width="12" customWidth="1" style="30" min="10" max="10"/>
+    <col width="14" customWidth="1" style="30" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1589,7 +1797,7 @@
   <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="145" customWidth="1" min="1" max="1"/>
+    <col width="145" customWidth="1" style="30" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1992,7 +2200,7 @@
   <dimension ref="A1:A86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="145" customWidth="1" min="1" max="1"/>
+    <col width="145" customWidth="1" style="30" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Split CZ26011062 into two declarations by transit MRN
JSD 1 now covers the whole 40' MRN (MRSU2171077, GW 26,600 kg) and
JSD 2 the whole 20' MRN (MRKU8681136, GW 12,130 kg), replacing the
earlier paid/free-of-charge split.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVghCknMruivM8JHkAAeLW
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
+++ b/output/HS_Code_Summary_Area_Four_Industries_CZ26011062.xlsx
@@ -874,23 +874,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="30" min="1" max="1"/>
-    <col width="5" customWidth="1" style="30" min="2" max="2"/>
-    <col width="14" customWidth="1" style="30" min="3" max="3"/>
-    <col width="34" customWidth="1" style="30" min="4" max="4"/>
-    <col width="8" customWidth="1" style="30" min="5" max="5"/>
-    <col width="10" customWidth="1" style="30" min="6" max="6"/>
+    <col width="15" customWidth="1" style="30" min="1" max="1"/>
+    <col width="30" customWidth="1" style="30" min="2" max="2"/>
+    <col width="5" customWidth="1" style="30" min="3" max="3"/>
+    <col width="14" customWidth="1" style="30" min="4" max="4"/>
+    <col width="48" customWidth="1" style="30" min="5" max="5"/>
+    <col width="8" customWidth="1" style="30" min="6" max="6"/>
     <col width="10" customWidth="1" style="30" min="7" max="7"/>
-    <col width="11" customWidth="1" style="30" min="8" max="8"/>
+    <col width="7" customWidth="1" style="30" min="8" max="8"/>
     <col width="11" customWidth="1" style="30" min="9" max="9"/>
-    <col width="13" customWidth="1" style="30" min="10" max="10"/>
-    <col width="13" customWidth="1" style="30" min="11" max="11"/>
-    <col width="12" customWidth="1" style="30" min="12" max="12"/>
-    <col width="13" customWidth="1" style="30" min="13" max="13"/>
-    <col width="14" customWidth="1" style="30" min="14" max="14"/>
+    <col width="11" customWidth="1" style="30" min="10" max="10"/>
+    <col width="22" customWidth="1" style="30" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -901,170 +898,141 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>MRN / kontejner</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Pol.</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>HS kód (TARIC)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Položka zákazníka</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Obsah</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Listů</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Objem m³ (MTQ)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Beden</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>NW (kg)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>GW (kg)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Hodnota USD</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Základ CZK (orient.)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>A00 clo 7 % (CZK)</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>A30 AD 86,8 % (CZK)</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Celkem clo + AD (CZK)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>JSD 1 – fakturované zboží</t>
-        </is>
-      </c>
-      <c r="B2" s="16" t="n">
+          <t>JSD 1</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>MRN …23258J0 – 40' MRSU2171077</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="16" t="inlineStr">
+      <c r="D2" s="16" t="inlineStr">
         <is>
           <t>4412 39 00 30</t>
         </is>
       </c>
-      <c r="D2" s="16" t="inlineStr">
-        <is>
-          <t>30207943, 39200442, 21200058, 39201550</t>
-        </is>
-      </c>
-      <c r="E2" s="17" t="n">
-        <v>1968</v>
-      </c>
-      <c r="F2" s="18" t="n">
-        <v>54.026</v>
-      </c>
-      <c r="G2" s="16" t="n">
-        <v>25</v>
-      </c>
-      <c r="H2" s="19" t="n">
-        <v>35300</v>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>15×993×1993 (4 bedny), 15×225×910 (1), 18×1220×2440 (10)</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="n">
+        <v>1266</v>
+      </c>
+      <c r="G2" s="18" t="n">
+        <v>36.101</v>
+      </c>
+      <c r="H2" s="17" t="n">
+        <v>15</v>
       </c>
       <c r="I2" s="19" t="n">
-        <v>36050</v>
+        <v>23470</v>
       </c>
       <c r="J2" s="19" t="n">
-        <v>33650.84</v>
-      </c>
-      <c r="K2" s="17" t="n">
-        <v>719131</v>
-      </c>
-      <c r="L2" s="17" t="n">
-        <v>50339</v>
-      </c>
-      <c r="M2" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="17" t="n">
-        <v>50339</v>
+        <v>23920</v>
+      </c>
+      <c r="K2" s="19" t="n">
+        <v>20459.22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>JSD 1 – fakturované zboží</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
+          <t>JSD 1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>MRN …23258J0 – 40' MRSU2171077</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>4412 33 10 82</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>39201508 GM5-Deska 4 mm – 18 placených listů</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>0.143</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>(v 2 bednách s FOC)</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>91.04000000000001</v>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>GM5-Deska 4×993×1993 – 18 ks placených + 500 ks FREE OF CHARGE (2 bedny)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>518</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>4.101</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>93.13</v>
+        <v>2620</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>189</v>
-      </c>
-      <c r="K3" s="3" t="n">
-        <v>4039</v>
-      </c>
-      <c r="L3" s="3" t="n">
-        <v>283</v>
-      </c>
-      <c r="M3" s="3" t="n">
-        <v>3506</v>
-      </c>
-      <c r="N3" s="3" t="n">
-        <v>3789</v>
+        <v>2680</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>189,00 + FOC 5 250,00</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1076,392 +1044,170 @@
       <c r="B4" s="20" t="inlineStr"/>
       <c r="C4" s="20" t="inlineStr"/>
       <c r="D4" s="20" t="inlineStr"/>
-      <c r="E4" s="21" t="n">
-        <v>1986</v>
-      </c>
-      <c r="F4" s="22" t="n">
-        <v>54.169</v>
-      </c>
-      <c r="G4" s="20" t="n">
-        <v>25</v>
-      </c>
-      <c r="H4" s="23" t="n">
-        <v>35391.04</v>
+      <c r="E4" s="20" t="inlineStr"/>
+      <c r="F4" s="21" t="n">
+        <v>1784</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>40.202</v>
+      </c>
+      <c r="H4" s="21" t="n">
+        <v>17</v>
       </c>
       <c r="I4" s="23" t="n">
-        <v>36143.13</v>
+        <v>26090</v>
       </c>
       <c r="J4" s="23" t="n">
-        <v>33839.84</v>
-      </c>
-      <c r="K4" s="21" t="n">
-        <v>723170</v>
-      </c>
-      <c r="L4" s="21" t="n">
-        <v>50622</v>
-      </c>
-      <c r="M4" s="21" t="n">
-        <v>3506</v>
-      </c>
-      <c r="N4" s="21" t="n">
-        <v>54128</v>
+        <v>26600</v>
+      </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>20 648,22 + FOC 5 250,00</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>JSD 2 – FREE OF CHARGE</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>JSD 2</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>MRN …23252J5 – 20' MRKU8681136</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>4412 33 10 82</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>39201508 GM5-Deska 4 mm – 500 listů zdarma</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>500</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>3.958</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>2528.96</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>2586.87</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>5250</v>
-      </c>
-      <c r="K5" s="3" t="n">
-        <v>112194</v>
-      </c>
-      <c r="L5" s="3" t="n">
-        <v>7854</v>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>97385</v>
-      </c>
-      <c r="N5" s="3" t="n">
-        <v>105238</v>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>4412 39 00 30</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>15×993×1993 (3 bedny), 12×994×1994 (7)</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>702</v>
+      </c>
+      <c r="G5" s="18" t="n">
+        <v>17.925</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" s="19" t="n">
+        <v>11830</v>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>12130</v>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>13191.62</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>CELKEM ZÁSILKA</t>
+          <t>JSD 2 CELKEM</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr"/>
       <c r="C6" s="20" t="inlineStr"/>
       <c r="D6" s="20" t="inlineStr"/>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="20" t="inlineStr"/>
+      <c r="F6" s="21" t="n">
+        <v>702</v>
+      </c>
+      <c r="G6" s="22" t="n">
+        <v>17.925</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>11830</v>
+      </c>
+      <c r="J6" s="23" t="n">
+        <v>12130</v>
+      </c>
+      <c r="K6" s="23" t="n">
+        <v>13191.62</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>ZÁSILKA CELKEM</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr"/>
+      <c r="C7" s="20" t="inlineStr"/>
+      <c r="D7" s="20" t="inlineStr"/>
+      <c r="E7" s="20" t="inlineStr"/>
+      <c r="F7" s="21" t="n">
         <v>2486</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="G7" s="22" t="n">
         <v>58.127</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="H7" s="21" t="n">
         <v>27</v>
       </c>
-      <c r="H6" s="23" t="n">
+      <c r="I7" s="23" t="n">
         <v>37920</v>
       </c>
-      <c r="I6" s="23" t="n">
+      <c r="J7" s="23" t="n">
         <v>38730</v>
       </c>
-      <c r="J6" s="23" t="inlineStr">
+      <c r="K7" s="20" t="inlineStr">
         <is>
           <t>33 839,84 + FOC 5 250,00</t>
         </is>
       </c>
-      <c r="K6" s="21" t="n">
-        <v>835364</v>
-      </c>
-      <c r="L6" s="21" t="n">
-        <v>58476</v>
-      </c>
-      <c r="M6" s="21" t="n">
-        <v>100891</v>
-      </c>
-      <c r="N6" s="21" t="n">
-        <v>159366</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Poznámky:</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>• Rozdělení: JSD 1 = vše fakturované (transakční hodnota, součet = TOTAL faktury US $33 839,84); JSD 2 = 500 listů FREE OF CHARGE.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>• Hodnota FOC: 500 × $10,50 (cena stejné desky z faktury) = $5 250 – NUTNO POTVRDIT se zákazníkem.</t>
+          <t>• Rozdělení podle MRN: JSD 1 = celé MRN …23258J0 (GW 26 600), JSD 2 = celé MRN …23252J5 (GW 12 130).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>• CZK přepočteny stejným poměrem jako výpočet K. Lukianové u 18 listů ($189,00 → 4 039 CZK, tj. 21,37037 CZK/USD) – orientační.</t>
+          <t>• Obsah kontejnerů doklady neuvádějí – odvozeno z hmotností beden a objemů dle faktury (jediná kombinace dávající 12 130 kg a 17,925 m³ pro 20').</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>• FOB Qingdao: do základu je ještě třeba připočíst dopravu a pojištění do místa vstupu do EU – částky výše je NEOBSAHUJÍ.</t>
+          <t>• 500 ks FREE OF CHARGE (4412 33 10 82) jsou v JSD 1 – hodnota 5 250 USD (10,50 USD/ks) k potvrzení se zákazníkem.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>• Hmotnosti 4mm desky: packing list neuvádí rozdělení 18/500 (2 bedny po 259 listech), NW/GW rozpočteny poměrem počtu listů.</t>
+          <t>• 4412 33 10 82: clo 7 % (A00) + konečné AD clo 86,8 % (A30). 4412 39 00 30: clo 7 %, registrace dovozu dle 2026/1840.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>• Beden: 18 placených listů je fyzicky ve stejných 2 bednách jako FOC listy – bedny vykázány jen jednou (JSD 2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• AD clo uvádět zvlášť jako A30 (86,8 %), A00 je jen clo 7 %. DPH (B00) není zahrnuta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="29" t="inlineStr">
-        <is>
-          <t>ROZPAD HMOTNOSTÍ PODLE MRN / KONTEJNERŮ</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>JSD / položka</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr"/>
-      <c r="C18" s="1" t="inlineStr">
-        <is>
-          <t>HS kód</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr"/>
-      <c r="E18" s="1" t="inlineStr">
-        <is>
-          <t>GW – MRN …23252J5 (20' MRKU8681136)</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="inlineStr">
-        <is>
-          <t>NW – MRN …23252J5</t>
-        </is>
-      </c>
-      <c r="G18" s="1" t="inlineStr">
-        <is>
-          <t>GW – MRN …23258J0 (40' MRSU2171077)</t>
-        </is>
-      </c>
-      <c r="H18" s="1" t="inlineStr">
-        <is>
-          <t>NW – MRN …23258J0</t>
-        </is>
-      </c>
-      <c r="I18" s="1" t="inlineStr">
-        <is>
-          <t>GW celkem</t>
-        </is>
-      </c>
-      <c r="J18" s="1" t="inlineStr">
-        <is>
-          <t>NW celkem</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="31" t="inlineStr">
-        <is>
-          <t>JSD 1 / pol. 1</t>
-        </is>
-      </c>
-      <c r="B19" s="31" t="inlineStr"/>
-      <c r="C19" s="31" t="inlineStr">
-        <is>
-          <t>4412 39 00 30</t>
-        </is>
-      </c>
-      <c r="D19" s="31" t="inlineStr"/>
-      <c r="E19" s="32" t="n">
-        <v>12130</v>
-      </c>
-      <c r="F19" s="32" t="n">
-        <v>11830</v>
-      </c>
-      <c r="G19" s="32" t="n">
-        <v>23920</v>
-      </c>
-      <c r="H19" s="32" t="n">
-        <v>23470</v>
-      </c>
-      <c r="I19" s="32" t="n">
-        <v>36050</v>
-      </c>
-      <c r="J19" s="32" t="n">
-        <v>35300</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="31" t="inlineStr">
-        <is>
-          <t>JSD 1 / pol. 2 (18 ks)</t>
-        </is>
-      </c>
-      <c r="B20" s="31" t="inlineStr"/>
-      <c r="C20" s="31" t="inlineStr">
-        <is>
-          <t>4412 33 10 82</t>
-        </is>
-      </c>
-      <c r="D20" s="31" t="inlineStr"/>
-      <c r="E20" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="32" t="n">
-        <v>93.13</v>
-      </c>
-      <c r="H20" s="32" t="n">
-        <v>91.04000000000001</v>
-      </c>
-      <c r="I20" s="32" t="n">
-        <v>93.13</v>
-      </c>
-      <c r="J20" s="32" t="n">
-        <v>91.04000000000001</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>JSD 1 CELKEM</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr"/>
-      <c r="C21" s="10" t="inlineStr"/>
-      <c r="D21" s="10" t="inlineStr"/>
-      <c r="E21" s="13" t="n">
-        <v>12130</v>
-      </c>
-      <c r="F21" s="13" t="n">
-        <v>11830</v>
-      </c>
-      <c r="G21" s="13" t="n">
-        <v>24013.13</v>
-      </c>
-      <c r="H21" s="13" t="n">
-        <v>23561.04</v>
-      </c>
-      <c r="I21" s="13" t="n">
-        <v>36143.13</v>
-      </c>
-      <c r="J21" s="13" t="n">
-        <v>35391.04</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="31" t="inlineStr">
-        <is>
-          <t>JSD 2 / pol. 1 (500 ks FOC)</t>
-        </is>
-      </c>
-      <c r="B22" s="31" t="inlineStr"/>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>4412 33 10 82</t>
-        </is>
-      </c>
-      <c r="D22" s="31" t="inlineStr"/>
-      <c r="E22" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="32" t="n">
-        <v>2586.87</v>
-      </c>
-      <c r="H22" s="32" t="n">
-        <v>2528.96</v>
-      </c>
-      <c r="I22" s="32" t="n">
-        <v>2586.87</v>
-      </c>
-      <c r="J22" s="32" t="n">
-        <v>2528.96</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>MRN CELKEM</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr"/>
-      <c r="C23" s="10" t="inlineStr"/>
-      <c r="D23" s="10" t="inlineStr"/>
-      <c r="E23" s="13" t="n">
-        <v>12130</v>
-      </c>
-      <c r="F23" s="13" t="n">
-        <v>11830</v>
-      </c>
-      <c r="G23" s="13" t="n">
-        <v>26600</v>
-      </c>
-      <c r="H23" s="13" t="n">
-        <v>26090</v>
-      </c>
-      <c r="I23" s="13" t="n">
-        <v>38730</v>
-      </c>
-      <c r="J23" s="13" t="n">
-        <v>37920</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Přiřazení beden ke kontejnerům je odvozeno z hmotností a objemů (doklady ho neuvádějí): 20' = 3 bedny 15×993×1993 + 7 beden 12×994×1994; 40' = zbytek vč. obou beden 4 mm.</t>
+          <t>• FOB Qingdao – do základu připočíst dopravu a pojištění do místa vstupu do EU.</t>
         </is>
       </c>
     </row>

</xml_diff>